<commit_message>
Stage 8 review fixes: D-010
</commit_message>
<xml_diff>
--- a/output/archive/QuenverellData/engagements/qv.25.086/docking/processed/dt8-pocket-water-hit-ranks-v2.xlsx
+++ b/output/archive/QuenverellData/engagements/qv.25.086/docking/processed/dt8-pocket-water-hit-ranks-v2.xlsx
@@ -154,7 +154,7 @@
   <commentList>
     <comment ref="B3" authorId="0" shapeId="0">
       <text>
-        <t>Check the chain labels against the client's file list before the next series is added</t>
+        <t>Consult coordinate provenance and the pocket-water assessment before extending the candidate set.</t>
       </text>
     </comment>
   </commentList>
@@ -169,7 +169,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Ranking is the design order used in the report; the water-removed runs are in the pocket waters sheet</t>
+        <t>Design identities and individual scores remain in the engagement source records.</t>
       </text>
     </comment>
   </commentList>
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -625,6 +625,16 @@
           <t>Item</t>
         </is>
       </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Source record</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -634,87 +644,67 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Client-supplied structures of the stress kinase, one per ligand series</t>
+          <t>Client-supplied in-house X-ray co-crystal coordinates</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Structures used as supplied; no re-refinement by Quenverell</t>
+          <t>Coordinates guided docking; provenance is in the client report</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Water retention</t>
+          <t>Pocket waters</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Water kept if it is conserved across the supplied structures and within the binding site</t>
+          <t>Conserved pocket-water assessment in the client report</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Waters seen in one structure only were treated as uncertain</t>
+          <t>Water assumptions affect docking interpretation</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Displaceable waters</t>
+          <t>Docking</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Waters near the solvent-facing edge scored as displaceable</t>
+          <t>Run settings and scores in the engagement records</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Assumption set by the medicinal chemistry question</t>
+          <t>Scores in kcal/mol support triage, not measured affinity</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Docking</t>
+          <t>Interpretation</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Ligands docked with conserved waters present and, separately, with them removed</t>
+          <t>Client report and ranked design record</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Both runs kept so the water assumption can be checked</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Interpretation</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Pose ranking is conditional on the water model</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Limits recorded in the report</t>
+          <t>A solvent-facing substitution opportunity was identified</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -727,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -739,20 +729,15 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Rank order</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Substitution vector</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Basis</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
@@ -761,66 +746,51 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>First</t>
+          <t>Design ranking</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Solvent-facing vector</t>
+          <t>Ranked design list retained with the engagement report</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Stable pose with conserved waters retained and removed</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Taken to the next chemistry cycle by Drelvessa</t>
+          <t>Consult the list for identities and ordering</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Second</t>
+          <t>Solvent-facing substitution</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Vector toward the hinge-side pocket</t>
+          <t>Opportunity identified by crystallography-based docking</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Pose depends on a single water</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Kept as back-up</t>
+          <t>Drelvessa carried it into its next chemistry cycle</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Third</t>
+          <t>Interpretation limit</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Other vectors</t>
+          <t>Ranking depends on receptor preparation and pocket-water assumptions</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Clash or unstable pose in more than one structure</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Not progressed</t>
+          <t>Experimental follow-up is needed to establish activity</t>
         </is>
       </c>
     </row>

</xml_diff>